<commit_message>
Remove authoring language and refresh final artifacts
</commit_message>
<xml_diff>
--- a/artifacts/关键标准答案.xlsx
+++ b/artifacts/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="Rba0e9e8525784413"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Re947d9b7786948ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Rb21a921cec384cc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R062b862acea44ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R126a00097f39437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R5c60fd53c08440b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Rfe145286cd194557"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Rb198069531804208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rbb4d4d686b774696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R030e3f5c1742436e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -935,7 +935,7 @@
         <x:v>路径中间对象</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>可保留额外候选路径或调试索引，但不得进入Reference交付</x:v>
+        <x:v>可保留额外候选路径或调试索引，但不得进入正式交付</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
         <x:v>device_path中的最佳路径及其深度和分数</x:v>

</xml_diff>